<commit_message>
Refocus agent workspace on source verification, review decisions and extraction accuracy
</commit_message>
<xml_diff>
--- a/samples/converted/01_invoice_register.xlsx
+++ b/samples/converted/01_invoice_register.xlsx
@@ -12,9 +12,11 @@
     <sheet name="Validation" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Evidence" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Corrections" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Page coverage" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Run log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Overview'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table 1'!$A$1:$P$32</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Table 1'!$1:$1</definedName>
@@ -24,6 +26,10 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Evidence'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Corrections'!$A$1:$F$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Corrections'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Page coverage'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Page coverage'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Run log'!$A$1:$D$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Run log'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -85,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -99,6 +105,9 @@
     <xf numFmtId="165" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="4" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -106,6 +115,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -504,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -592,7 +604,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -615,36 +627,106 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>LedgerLens 1.0 · PyMuPDF + RapidOCR (PP-OCR / ONNX)</t>
+          <t>LedgerLens 1.1 · PyMuPDF + RapidOCR (PP-OCR / ONNX)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Interpretation</t>
+          <t>Review status</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>OCR recognition scores are not measured extraction accuracy. Review all findings.</t>
+          <t>Draft — review pending</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Pages with extracted tables</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>3 / 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Validation errors</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Validation warnings</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Rows with source evidence</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Review note</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Review completed (UTC)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>OCR recognition scores are not measured extraction accuracy. Review all findings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Pages without extracted tables are explicitly flagged. No guarantee for arbitrary layouts.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -781,19 +863,19 @@
       <c r="E2" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="G2" s="6" t="n">
+      <c r="G2" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="I2" s="6" t="n">
         <v>4.4</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="6" t="n">
         <v>48.4</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -827,7 +909,7 @@
           <t>INV-0002</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
+      <c r="B3" s="8" t="n">
         <v>46298</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -840,22 +922,22 @@
           <t>North</t>
         </is>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="G3" s="9" t="n">
+      <c r="G3" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="10" t="n">
         <v>7.2</v>
       </c>
-      <c r="J3" s="8" t="n">
+      <c r="J3" s="10" t="n">
         <v>79.2</v>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -905,19 +987,19 @@
       <c r="E4" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="G4" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="6" t="n">
         <v>104</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I4" s="6" t="n">
         <v>10.4</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="6" t="n">
         <v>114.4</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -951,7 +1033,7 @@
           <t>INV-0004</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="8" t="n">
         <v>46300</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -964,22 +1046,22 @@
           <t>West</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="G5" s="9" t="n">
+      <c r="G5" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="10" t="n">
         <v>140</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="J5" s="8" t="n">
+      <c r="J5" s="10" t="n">
         <v>154</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -1029,19 +1111,19 @@
       <c r="E6" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="6" t="n">
         <v>180</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I6" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="6" t="n">
         <v>198</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1075,7 +1157,7 @@
           <t>INV-0006</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="8" t="n">
         <v>46302</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1088,22 +1170,22 @@
           <t>East</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="10" t="n">
         <v>224</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="10" t="n">
         <v>22.4</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="10" t="n">
         <v>246.4</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1153,19 +1235,19 @@
       <c r="E8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="6" t="n">
         <v>3.4</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="6" t="n">
         <v>37.4</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1199,7 +1281,7 @@
           <t>INV-0008</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="8" t="n">
         <v>46304</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1212,22 +1294,22 @@
           <t>North</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="10" t="n">
         <v>36</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G9" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="10" t="n">
         <v>7.2</v>
       </c>
-      <c r="J9" s="8" t="n">
+      <c r="J9" s="10" t="n">
         <v>79.2</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1277,19 +1359,19 @@
       <c r="E10" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="6" t="n">
         <v>114</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="I10" s="6" t="n">
         <v>11.4</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="6" t="n">
         <v>125.4</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1323,7 +1405,7 @@
           <t>INV-0010</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="8" t="n">
         <v>46306</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1336,22 +1418,22 @@
           <t>West</t>
         </is>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F11" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="G11" s="9" t="n">
+      <c r="G11" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="10" t="n">
         <v>160</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="10" t="n">
         <v>16</v>
       </c>
-      <c r="J11" s="8" t="n">
+      <c r="J11" s="10" t="n">
         <v>176</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1401,19 +1483,19 @@
       <c r="E12" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="I12" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="J12" s="6" t="n">
         <v>231</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1447,7 +1529,7 @@
           <t>INV-0012</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="8" t="n">
         <v>46308</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1460,22 +1542,22 @@
           <t>East</t>
         </is>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F13" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="G13" s="9" t="n">
+      <c r="G13" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="10" t="n">
         <v>264</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="I13" s="10" t="n">
         <v>26.4</v>
       </c>
-      <c r="J13" s="8" t="n">
+      <c r="J13" s="10" t="n">
         <v>290.4</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -1525,19 +1607,19 @@
       <c r="E14" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="G14" s="6" t="n">
+      <c r="G14" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H14" s="5" t="n">
+      <c r="H14" s="6" t="n">
         <v>322</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="I14" s="6" t="n">
         <v>32.2</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="J14" s="6" t="n">
         <v>354.2</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1571,7 +1653,7 @@
           <t>INV-0014</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="8" t="n">
         <v>46310</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1584,22 +1666,22 @@
           <t>North</t>
         </is>
       </c>
-      <c r="E15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="8" t="n">
+      <c r="E15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G15" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="10" t="n">
         <v>4.8</v>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="10" t="n">
         <v>52.8</v>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -1649,19 +1731,19 @@
       <c r="E16" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="G16" s="6" t="n">
+      <c r="G16" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="H16" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="6" t="n">
         <v>110</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1695,7 +1777,7 @@
           <t>INV-0016</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="8" t="n">
         <v>46312</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1708,22 +1790,22 @@
           <t>West</t>
         </is>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F17" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G17" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="10" t="n">
         <v>156</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="I17" s="10" t="n">
         <v>15.6</v>
       </c>
-      <c r="J17" s="8" t="n">
+      <c r="J17" s="10" t="n">
         <v>171.6</v>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -1773,19 +1855,19 @@
       <c r="E18" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="G18" s="6" t="n">
+      <c r="G18" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H18" s="6" t="n">
         <v>216</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="6" t="n">
         <v>21.6</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J18" s="6" t="n">
         <v>237.6</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1819,7 +1901,7 @@
           <t>INV-0018</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="8" t="n">
         <v>46314</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1832,22 +1914,22 @@
           <t>East</t>
         </is>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F19" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G19" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="10" t="n">
         <v>280</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="I19" s="10" t="n">
         <v>28</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="10" t="n">
         <v>308</v>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1897,19 +1979,19 @@
       <c r="E20" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F20" s="5" t="n">
+      <c r="F20" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="G20" s="6" t="n">
+      <c r="G20" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="H20" s="6" t="n">
         <v>348</v>
       </c>
-      <c r="I20" s="5" t="n">
+      <c r="I20" s="6" t="n">
         <v>34.8</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="J20" s="6" t="n">
         <v>382.8</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1943,7 +2025,7 @@
           <t>INV-0020</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="8" t="n">
         <v>46316</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1956,22 +2038,22 @@
           <t>North</t>
         </is>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F21" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="G21" s="9" t="n">
+      <c r="G21" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="10" t="n">
         <v>420</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="I21" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="J21" s="8" t="n">
+      <c r="J21" s="10" t="n">
         <v>462</v>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -2021,19 +2103,19 @@
       <c r="E22" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="G22" s="6" t="n">
+      <c r="G22" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="H22" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="I22" s="6" t="n">
         <v>6.2</v>
       </c>
-      <c r="J22" s="5" t="n">
+      <c r="J22" s="6" t="n">
         <v>68.2</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2067,7 +2149,7 @@
           <t>INV-0022</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="8" t="n">
         <v>46318</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -2080,22 +2162,22 @@
           <t>West</t>
         </is>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E23" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="G23" s="9" t="n">
+      <c r="G23" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="I23" s="8" t="n">
+      <c r="I23" s="10" t="n">
         <v>12.8</v>
       </c>
-      <c r="J23" s="8" t="n">
+      <c r="J23" s="10" t="n">
         <v>140.8</v>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -2145,19 +2227,19 @@
       <c r="E24" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="5" t="n">
+      <c r="F24" s="6" t="n">
         <v>66</v>
       </c>
-      <c r="G24" s="6" t="n">
+      <c r="G24" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H24" s="5" t="n">
+      <c r="H24" s="6" t="n">
         <v>198</v>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="I24" s="6" t="n">
         <v>19.8</v>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="J24" s="6" t="n">
         <v>217.8</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2191,7 +2273,7 @@
           <t>INV-0024</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="8" t="n">
         <v>46320</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -2204,22 +2286,22 @@
           <t>East</t>
         </is>
       </c>
-      <c r="E25" s="8" t="n">
+      <c r="E25" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="F25" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="G25" s="9" t="n">
+      <c r="G25" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="H25" s="10" t="n">
         <v>272</v>
       </c>
-      <c r="I25" s="8" t="n">
+      <c r="I25" s="10" t="n">
         <v>27.2</v>
       </c>
-      <c r="J25" s="8" t="n">
+      <c r="J25" s="10" t="n">
         <v>299.2</v>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -2269,19 +2351,19 @@
       <c r="E26" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F26" s="5" t="n">
+      <c r="F26" s="6" t="n">
         <v>70</v>
       </c>
-      <c r="G26" s="6" t="n">
+      <c r="G26" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H26" s="5" t="n">
+      <c r="H26" s="6" t="n">
         <v>350</v>
       </c>
-      <c r="I26" s="5" t="n">
+      <c r="I26" s="6" t="n">
         <v>35</v>
       </c>
-      <c r="J26" s="5" t="n">
+      <c r="J26" s="6" t="n">
         <v>385</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2315,7 +2397,7 @@
           <t>INV-0026</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n">
+      <c r="B27" s="8" t="n">
         <v>46322</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -2328,22 +2410,22 @@
           <t>North</t>
         </is>
       </c>
-      <c r="E27" s="8" t="n">
+      <c r="E27" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="F27" s="8" t="n">
+      <c r="F27" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="G27" s="9" t="n">
+      <c r="G27" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="10" t="n">
         <v>432</v>
       </c>
-      <c r="I27" s="8" t="n">
+      <c r="I27" s="10" t="n">
         <v>43.2</v>
       </c>
-      <c r="J27" s="8" t="n">
+      <c r="J27" s="10" t="n">
         <v>475.2</v>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -2393,19 +2475,19 @@
       <c r="E28" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="F28" s="5" t="n">
+      <c r="F28" s="6" t="n">
         <v>74</v>
       </c>
-      <c r="G28" s="6" t="n">
+      <c r="G28" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H28" s="5" t="n">
+      <c r="H28" s="6" t="n">
         <v>518</v>
       </c>
-      <c r="I28" s="5" t="n">
+      <c r="I28" s="6" t="n">
         <v>51.8</v>
       </c>
-      <c r="J28" s="5" t="n">
+      <c r="J28" s="6" t="n">
         <v>569.8</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2439,7 +2521,7 @@
           <t>INV-0028</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B29" s="8" t="n">
         <v>46296</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -2452,22 +2534,22 @@
           <t>West</t>
         </is>
       </c>
-      <c r="E29" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="8" t="n">
+      <c r="E29" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="G29" s="9" t="n">
+      <c r="G29" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I29" s="8" t="n">
+      <c r="I29" s="10" t="n">
         <v>7.6</v>
       </c>
-      <c r="J29" s="8" t="n">
+      <c r="J29" s="10" t="n">
         <v>83.59999999999999</v>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -2517,19 +2599,19 @@
       <c r="E30" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F30" s="5" t="n">
+      <c r="F30" s="6" t="n">
         <v>78</v>
       </c>
-      <c r="G30" s="6" t="n">
+      <c r="G30" s="7" t="n">
         <v>0.1</v>
       </c>
-      <c r="H30" s="5" t="n">
+      <c r="H30" s="6" t="n">
         <v>156</v>
       </c>
-      <c r="I30" s="5" t="n">
+      <c r="I30" s="6" t="n">
         <v>15.6</v>
       </c>
-      <c r="J30" s="5" t="n">
+      <c r="J30" s="6" t="n">
         <v>171.6</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2563,7 +2645,7 @@
           <t>INV-0030</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B31" s="8" t="n">
         <v>46298</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2576,22 +2658,22 @@
           <t>East</t>
         </is>
       </c>
-      <c r="E31" s="8" t="n">
+      <c r="E31" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F31" s="8" t="n">
+      <c r="F31" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="G31" s="9" t="n">
+      <c r="G31" s="11" t="n">
         <v>0.1</v>
       </c>
-      <c r="H31" s="8" t="n">
+      <c r="H31" s="10" t="n">
         <v>240</v>
       </c>
-      <c r="I31" s="8" t="n">
+      <c r="I31" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="J31" s="8" t="n">
+      <c r="J31" s="10" t="n">
         <v>264</v>
       </c>
       <c r="K31" s="3" t="inlineStr">
@@ -2633,13 +2715,13 @@
       </c>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="5" t="n">
+      <c r="H32" s="6" t="n">
         <v>5940</v>
       </c>
-      <c r="I32" s="5" t="n">
+      <c r="I32" s="6" t="n">
         <v>594</v>
       </c>
-      <c r="J32" s="5" t="n">
+      <c r="J32" s="6" t="n">
         <v>6534</v>
       </c>
       <c r="K32" s="2" t="inlineStr"/>
@@ -3599,4 +3681,389 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Extraction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Table fragments</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Data rows (page estimate)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Seconds</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Attempts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>extracted</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>native</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Time (UTC)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Stage</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.142541+00:00</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Opened source document</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.157503+00:00</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Selected native text extraction</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.232591+00:00</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Extracted table fragments</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.246170+00:00</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Selected native text extraction</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.316966+00:00</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Extracted table fragments</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.318968+00:00</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>inspect</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Selected native text extraction</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.389716+00:00</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>extract</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Extracted table fragments</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.389716+00:00</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>align</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Matching table schemas and continuation pages</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.389716+00:00</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>validate</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Checking totals, arithmetic, balances and table integrity</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-15T06:05:37.389716+00:00</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Extraction complete; human review is pending</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Keep native PDF recognition scores blank in exported workbooks
</commit_message>
<xml_diff>
--- a/samples/converted/01_invoice_register.xlsx
+++ b/samples/converted/01_invoice_register.xlsx
@@ -899,9 +899,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P2" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -961,9 +959,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P3" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P3" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -1023,9 +1019,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P4" s="2" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1085,9 +1079,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P5" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P5" s="3" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -1147,9 +1139,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P6" s="2" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1209,9 +1199,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P7" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P7" s="3" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -1271,9 +1259,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P8" s="2" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1333,9 +1319,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P9" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P9" s="3" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -1395,9 +1379,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P10" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P10" s="2" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -1457,9 +1439,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P11" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P11" s="3" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1519,9 +1499,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P12" s="2" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -1581,9 +1559,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P13" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P13" s="3" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -1643,9 +1619,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P14" s="2" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -1705,9 +1679,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P15" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P15" s="3" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1767,9 +1739,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P16" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P16" s="2" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -1829,9 +1799,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P17" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P17" s="3" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -1891,9 +1859,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P18" s="2" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -1953,9 +1919,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P19" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P19" s="3" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -2015,9 +1979,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P20" s="2" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -2077,9 +2039,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P21" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P21" s="3" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -2139,9 +2099,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P22" s="2" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -2201,9 +2159,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P23" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P23" s="3" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
@@ -2263,9 +2219,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P24" s="2" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -2325,9 +2279,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P25" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P25" s="3" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
@@ -2387,9 +2339,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P26" s="2" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -2449,9 +2399,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P27" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P27" s="3" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
@@ -2511,9 +2459,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P28" s="2" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -2573,9 +2519,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P29" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P29" s="3" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -2635,9 +2579,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P30" s="2" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
@@ -2697,9 +2639,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P31" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="P31" s="3" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -2737,9 +2677,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="P32" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P32" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P32"/>
@@ -2896,9 +2834,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="n">
@@ -2920,9 +2856,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F3" s="3" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -2944,9 +2878,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F4" s="2" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -2968,9 +2900,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F5" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F5" s="3" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -2992,9 +2922,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F6" s="2" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="n">
@@ -3016,9 +2944,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F7" s="3" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -3040,9 +2966,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F8" s="2" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="n">
@@ -3064,9 +2988,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F9" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F9" s="3" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -3088,9 +3010,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F10" s="2" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="n">
@@ -3112,9 +3032,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F11" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F11" s="3" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -3136,9 +3054,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F12" s="2" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="n">
@@ -3160,9 +3076,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F13" s="3" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -3184,9 +3098,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F14" s="2" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="3" t="n">
@@ -3208,9 +3120,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F15" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F15" s="3" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -3232,9 +3142,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F16" s="2" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="3" t="n">
@@ -3256,9 +3164,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F17" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F17" s="3" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -3280,9 +3186,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F18" s="2" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="3" t="n">
@@ -3304,9 +3208,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F19" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F19" s="3" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -3328,9 +3230,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F20" s="2" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="3" t="n">
@@ -3352,9 +3252,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F21" s="3" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -3376,9 +3274,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="3" t="n">
@@ -3400,9 +3296,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F23" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F23" s="3" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -3424,9 +3318,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F24" s="2" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="3" t="n">
@@ -3448,9 +3340,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F25" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F25" s="3" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -3472,9 +3362,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="3" t="n">
@@ -3496,9 +3384,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F27" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F27" s="3" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="n">
@@ -3520,9 +3406,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F28" s="2" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="3" t="n">
@@ -3544,9 +3428,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F29" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F29" s="3" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -3568,9 +3450,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F30" s="2" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="3" t="n">
@@ -3592,9 +3472,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F31" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="F31" s="3" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -3616,9 +3494,7 @@
           <t>Native PDF · grid</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="F32" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F32"/>

</xml_diff>

<commit_message>
Rename DamnLens AI Agent and strengthen judge setup and extraction accuracy
</commit_message>
<xml_diff>
--- a/samples/converted/01_invoice_register.xlsx
+++ b/samples/converted/01_invoice_register.xlsx
@@ -526,7 +526,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LedgerLens extraction report</t>
+          <t>DamnLens AI Agent extraction report</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -615,7 +615,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>9600d2184cd663da6698d3e4eae4a8a8634d62abcee18e7b264623805b6bbd2e</t>
+          <t>2504d1c047c23512733b3e08a8af778c51b57b8a50ee7d6353c075566ebb3fc2</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>LedgerLens 1.1 · PyMuPDF + RapidOCR (PP-OCR / ONNX)</t>
+          <t>DamnLens AI Agent 1.2 · PyMuPDF + RapidOCR (PP-OCR / ONNX)</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3659,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -3688,7 +3688,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.142541+00:00</t>
+          <t>2026-10-15T06:39:50.105645+00:00</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.157503+00:00</t>
+          <t>2026-10-15T06:39:50.118611+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.232591+00:00</t>
+          <t>2026-10-15T06:39:50.182983+00:00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -3806,7 +3806,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.246170+00:00</t>
+          <t>2026-10-15T06:39:50.192272+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3826,7 +3826,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.316966+00:00</t>
+          <t>2026-10-15T06:39:50.251292+00:00</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3846,7 +3846,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.318968+00:00</t>
+          <t>2026-10-15T06:39:50.262076+00:00</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.389716+00:00</t>
+          <t>2026-10-15T06:39:50.332142+00:00</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3886,7 +3886,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.389716+00:00</t>
+          <t>2026-10-15T06:39:50.332142+00:00</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3904,7 +3904,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.389716+00:00</t>
+          <t>2026-10-15T06:39:50.332142+00:00</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3922,7 +3922,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:05:37.389716+00:00</t>
+          <t>2026-10-15T06:39:50.332142+00:00</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Improve complex table reconstruction and verified page recovery
</commit_message>
<xml_diff>
--- a/samples/converted/01_invoice_register.xlsx
+++ b/samples/converted/01_invoice_register.xlsx
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.24</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -627,7 +627,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DamnLens AI Agent 1.2 · PyMuPDF + RapidOCR (PP-OCR / ONNX)</t>
+          <t>DamnLens AI Agent 1.3 · PyMuPDF + RapidOCR (PP-OCR / ONNX)</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3630,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -3659,7 +3659,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -3688,7 +3688,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.105645+00:00</t>
+          <t>2026-10-15T07:48:13.877763+00:00</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.118611+00:00</t>
+          <t>2026-10-15T07:48:13.884692+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.182983+00:00</t>
+          <t>2026-10-15T07:48:13.994854+00:00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -3806,7 +3806,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.192272+00:00</t>
+          <t>2026-10-15T07:48:13.996854+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3826,7 +3826,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.251292+00:00</t>
+          <t>2026-10-15T07:48:14.104918+00:00</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3846,7 +3846,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.262076+00:00</t>
+          <t>2026-10-15T07:48:14.106918+00:00</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.332142+00:00</t>
+          <t>2026-10-15T07:48:14.220641+00:00</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3886,7 +3886,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.332142+00:00</t>
+          <t>2026-10-15T07:48:14.220641+00:00</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3904,7 +3904,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.332142+00:00</t>
+          <t>2026-10-15T07:48:14.225101+00:00</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3922,7 +3922,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T06:39:50.332142+00:00</t>
+          <t>2026-10-15T07:48:14.230100+00:00</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Strengthen public scan accuracy and preserve OCR disagreements for review
</commit_message>
<xml_diff>
--- a/samples/converted/01_invoice_register.xlsx
+++ b/samples/converted/01_invoice_register.xlsx
@@ -627,7 +627,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DamnLens AI Agent 1.3 · PyMuPDF + RapidOCR (PP-OCR / ONNX)</t>
+          <t>DamnLens AI Agent 1.4 · PyMuPDF + RapidOCR (PP-OCRv3/v5 / ONNX)</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3688,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:13.877763+00:00</t>
+          <t>2026-10-15T08:42:18.538856+00:00</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3766,7 +3766,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:13.884692+00:00</t>
+          <t>2026-10-15T08:42:18.546889+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3786,7 +3786,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:13.994854+00:00</t>
+          <t>2026-10-15T08:42:18.655971+00:00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -3806,7 +3806,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:13.996854+00:00</t>
+          <t>2026-10-15T08:42:18.655971+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3826,7 +3826,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:14.104918+00:00</t>
+          <t>2026-10-15T08:42:18.766267+00:00</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3846,7 +3846,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:14.106918+00:00</t>
+          <t>2026-10-15T08:42:18.768922+00:00</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3866,7 +3866,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:14.220641+00:00</t>
+          <t>2026-10-15T08:42:18.884915+00:00</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3886,7 +3886,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:14.220641+00:00</t>
+          <t>2026-10-15T08:42:18.884915+00:00</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3904,7 +3904,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:14.225101+00:00</t>
+          <t>2026-10-15T08:42:18.888397+00:00</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3922,7 +3922,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T07:48:14.230100+00:00</t>
+          <t>2026-10-15T08:42:18.888397+00:00</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Add local and Gemini-assisted AI workflows with bounded source review
</commit_message>
<xml_diff>
--- a/samples/converted/01_invoice_register.xlsx
+++ b/samples/converted/01_invoice_register.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Run log" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$B$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Overview'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table 1'!$A$1:$P$32</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Table 1'!$1:$1</definedName>
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.35</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -634,31 +634,31 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Review status</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Draft — review pending</t>
+          <t>local</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Pages with extracted tables</t>
+          <t>Gemini model</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3 / 3</t>
+          <t>Not used</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Validation errors</t>
+          <t>Gemini request attempts</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -668,7 +668,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Validation warnings</t>
+          <t>Gemini reported total tokens</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -678,55 +678,111 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Rows with source evidence</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>31</v>
+          <t>Gemini interpretation</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>No external AI API requests.</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Review note</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr"/>
+          <t>Review status</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Draft — review pending</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Review completed (UTC)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr"/>
+          <t>Pages with extracted tables</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>3 / 3</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Interpretation</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>OCR recognition scores are not measured extraction accuracy. Review all findings.</t>
-        </is>
+          <t>Validation errors</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>Validation warnings</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Rows with source evidence</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Review note</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Review completed (UTC)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Interpretation</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>OCR recognition scores are not measured extraction accuracy. Review all findings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Pages without extracted tables are explicitly flagged. No guarantee for arbitrary layouts.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B19"/>
+  <autoFilter ref="A1:B24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -3630,7 +3686,7 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -3688,7 +3744,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -3748,7 +3804,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.538856+00:00</t>
+          <t>2026-10-15T09:24:51.319348+00:00</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3766,7 +3822,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.546889+00:00</t>
+          <t>2026-10-15T09:24:51.324186+00:00</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -3786,7 +3842,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.655971+00:00</t>
+          <t>2026-10-15T09:24:51.431584+00:00</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -3806,7 +3862,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.655971+00:00</t>
+          <t>2026-10-15T09:24:51.434129+00:00</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3826,7 +3882,7 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.766267+00:00</t>
+          <t>2026-10-15T09:24:51.540372+00:00</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3846,7 +3902,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.768922+00:00</t>
+          <t>2026-10-15T09:24:51.542537+00:00</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3866,7 +3922,7 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.884915+00:00</t>
+          <t>2026-10-15T09:24:51.651703+00:00</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3886,7 +3942,7 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.884915+00:00</t>
+          <t>2026-10-15T09:24:51.651703+00:00</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3904,7 +3960,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.888397+00:00</t>
+          <t>2026-10-15T09:24:51.654806+00:00</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3922,7 +3978,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2026-10-15T08:42:18.888397+00:00</t>
+          <t>2026-10-15T09:24:51.658159+00:00</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">

</xml_diff>